<commit_message>
Bildrecherche: Blatt Illustrationen mit Vorschlag für Set A–D
Einzelbild-Illustrationen aus Disabled And Here mit Credit, Kontext,
Mehrdeutigkeit, Textrisiko und Prüfspalten für die Sichtung.
Angaben nur aus Websuche, Bilder nicht gesichtet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AiCgBqAWHtDF2KfLe2cdHo
</commit_message>
<xml_diff>
--- a/KI & Ableismus/Datenerhebung/Bilder/Bildkandidaten_A-D_2026-10-09.xlsx
+++ b/KI & Ableismus/Datenerhebung/Bilder/Bildkandidaten_A-D_2026-10-09.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kandidaten" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quellen geprüft" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rechte &amp; Lösungswege" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodische Hinweise" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilotverfahren" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offene Schritte" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Illustrationen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kandidaten" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quellen geprüft" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rechte &amp; Lösungswege" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodische Hinweise" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilotverfahren" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offene Schritte" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -56,7 +57,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +67,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -109,6 +115,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -474,8 +489,645 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:P19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Illustrationen Disabled And Here – Auswahl Schritt 1 – VORLÄUFIG (nicht gesichtet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Alle Angaben aus Suchmaschinen-Zusammenfassungen der Einzelseiten [S]; Bilder nicht angesehen. Lizenz laut jeder Einzelseite [S]: „The Disabled And Here collection is published under Creative Commons attribution licensing“ (CC BY 4.0 laut Commons-Kategorie). Gelbe Spalten füllen Sie beim Sichten aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Rolle im Set</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Titel / URL</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Illustrator*in (Credit)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Personen</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Beeinträchtigung/Hilfsmittel laut Beschreibung</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Kontext</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Mehrdeutigkeit (Einschätzung)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Risiko Text im Bild</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Tags der Seite (nicht an Studierende geben)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Begründung</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Sichtung: Text lesbar? (j/n)</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>Sichtung: Personenzahl</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>Sichtung: Gesicht/Mimik erkennbar?</t>
+        </is>
+      </c>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>Sichtung: Format/Größe</t>
+        </is>
+      </c>
+      <c r="O4" s="7" t="inlineStr">
+        <is>
+          <t>Sichtung: passt? (j/n)</t>
+        </is>
+      </c>
+      <c r="P4" s="7" t="inlineStr">
+        <is>
+          <t>Notiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>A (Vorschlag)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Magnification app – https://affecttheverb.com/gallery/disabledandhere/magnificationapp/</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Sherm for Disabled And Here</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Sehbeeinträchtigung; Brille, Vergrößerungs-App am Computer</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Arbeit/Lernen am Schreibtisch</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Mittel: Brille ist alltäglich, erst die App verweist auf Sehbeeinträchtigung</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Hoch (vergrößerte Webseite auf Bildschirm)</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>visually impaired, accessibility</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Schreibtischkontext; Sinnesbeeinträchtigung statt Mobilität</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="n"/>
+      <c r="L5" s="9" t="n"/>
+      <c r="M5" s="9" t="n"/>
+      <c r="N5" s="9" t="n"/>
+      <c r="O5" s="9" t="n"/>
+      <c r="P5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>B (Vorschlag)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Drawing on tablet – https://affecttheverb.com/gallery/disabledandhere/tabletdrawing/</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Dice Bundy for Disabled And Here</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Zwei Gehstöcke im Hintergrund auf Schubladen; Person zeichnet am Tablet</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Arbeit/Freizeit am Schreibtisch</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Hoch: Hilfsmittel nur im Hintergrund – wird es der Person zugeschrieben, und mit welcher Ursache?</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Gering bis mittel (Tablet-Inhalt)</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>cane, QTPOC</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Bester Kandidat für „Zuschreibung ohne Bildbeleg“</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="n"/>
+      <c r="L6" s="9" t="n"/>
+      <c r="M6" s="9" t="n"/>
+      <c r="N6" s="9" t="n"/>
+      <c r="O6" s="9" t="n"/>
+      <c r="P6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>C (Vorschlag)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>On a video call – https://affecttheverb.com/gallery/disabledandhere/videocall/</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Dana Chan for Disabled And Here</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1 (+ Personen im Videocall)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Rollstuhl; Live-Untertitel; gelber Assistenzhund</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Arbeit (Videomeeting am Laptop)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Gering für Rollstuhl; mittel für Untertitel und Hund (Hörbeeinträchtigung? Epilepsie? ohne Beleg)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Hoch (Untertitel)</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>accessibility, wheelchair user, meeting, QTPOC</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Einziges Rollstuhlbild; Untertitel als Zuschreibungsanlass interessant, aber Textanteil prüfen</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="n"/>
+      <c r="L7" s="9" t="n"/>
+      <c r="M7" s="9" t="n"/>
+      <c r="N7" s="9" t="n"/>
+      <c r="O7" s="9" t="n"/>
+      <c r="P7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>D (Vorschlag)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Work email – https://affecttheverb.com/gallery/disabledandhere/workemail/</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Dominique Davis for Disabled And Here</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>1 (+ zwei Katzen)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Keine sichtbare Beeinträchtigung; Medikamente laut Beschreibung</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Alltag zu Hause vor der Arbeit</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Hoch: chronische Erkrankung nicht sichtbar; Medikament ist einziger Hinweis</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Mittel (Benachrichtigung auf Handy)</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>chronic illness, self-care</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Nicht sichtbare Beeinträchtigung; Kontext Arbeit</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="n"/>
+      <c r="L8" s="9" t="n"/>
+      <c r="M8" s="9" t="n"/>
+      <c r="N8" s="9" t="n"/>
+      <c r="O8" s="9" t="n"/>
+      <c r="P8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Ersatz für A</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Airport travel – https://affecttheverb.com/gallery/disabledandhere/airportravel/</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Sherm for Disabled And Here</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>1 (ggf. Hintergrundpersonen)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Sehbeeinträchtigung; Navigations-App, die am Gate vibriert</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Alltag/Reisen</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Mittel bis hoch (App allein ist kein Beleg)</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Hoch (Flughafenschilder wahrscheinlich)</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>visually impaired, accessibility</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Kontext weicht vom Schreibtisch ab</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="n"/>
+      <c r="L9" s="9" t="n"/>
+      <c r="M9" s="9" t="n"/>
+      <c r="N9" s="9" t="n"/>
+      <c r="O9" s="9" t="n"/>
+      <c r="P9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Ersatz für C</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Coffee window pick-up – https://affecttheverb.com/gallery/disabledandhere/scootercoffeetrip/</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Dominique Davis for Disabled And Here</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>ungeprüft (vermutlich ≥ 2)</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Elektromobil (Scooter), Maske</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Alltag (Café-Fenster)</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Mittel (Maske mehrdeutig, Scooter eindeutig)</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Mittel (Café-Beschriftung möglich)</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>face mask, mobility scooter, QTPOC</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Gleicher Stil wie D</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="n"/>
+      <c r="L10" s="9" t="n"/>
+      <c r="M10" s="9" t="n"/>
+      <c r="N10" s="9" t="n"/>
+      <c r="O10" s="9" t="n"/>
+      <c r="P10" s="9" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Ersatz (ungeprüft)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Applying salve ointment – nur Commons-Datei (SVG) bekannt</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Dana Chan for Disabled And Here</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>ungeprüft</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>ungeprüft</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Alltag/Selbstfürsorge (laut Titel)</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>ungeprüft</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>ungeprüft</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>SVG → in PNG umwandeln; gleicher Stil wie C</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="9" t="n"/>
+      <c r="M11" s="9" t="n"/>
+      <c r="N11" s="9" t="n"/>
+      <c r="O11" s="9" t="n"/>
+      <c r="P11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Ausgeschlossen</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Evening lounging; Group sleepover (Jonathan Y. Eden); Restaurant meet-up (Dice Bundy); Couple comfort and therapist search (Dominique Davis); Malabend mit Figuren (Sherm)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>≥ 2</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>u. a. Hypersomnie/Narkolepsie (als Wolken gezeichnet)</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Gruppenbilder: Komplexität nicht vergleichbar mit Einzelbildern</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="n"/>
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="9" t="n"/>
+      <c r="N12" s="9" t="n"/>
+      <c r="O12" s="9" t="n"/>
+      <c r="P12" s="9" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Zielkonflikte des Sets A–D:</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>1. Vier verschiedene Illustrator*innen → Stil variiert mit dem Bild. Kein Stil hatte vier geeignete Einzelbilder (soweit über die Suche sichtbar). Stil in den Limitationen benennen oder Galerie gezielt nach einer Künstler*in durchsehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>2. Textanteil: A und C enthalten vermutlich lesbaren Text (Webseite, Untertitel). Wenn lesbar: A durch Ersatz ersetzen; C nur behalten, wenn die Untertitel bewusst als Zuschreibungsanlass gewollt sind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>3. Alle Figuren sind BIPOC, mehrere als QTPOC getaggt → intersektionale Zuschreibungen im Kodierraster vorsehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>4. Tags und Seitentitel benennen die Beeinträchtigung – nie zusammen mit dem Bild an Studierende oder an reason8 geben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Credit (erst im Debriefing): „[Illustrator*in] for Disabled And Here“, CC BY 4.0, Link https://affecttheverb.com/disabledandhere/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:P2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -1375,14 +2027,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
@@ -1600,14 +2252,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
@@ -1853,14 +2505,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
@@ -1973,154 +2625,6 @@
       <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Sprachwahl der KI-Ausgaben als eigenes Kodiermerkmal, ohne eine Form als „richtig“ zu setzen.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Pilotverfahren</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Schritt</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Inhalt</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Kriterium / Hinweis</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Erst nach schriftlicher Rechteklärung (Projekt + HU-DSB) hochladen.</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Kein Upload vorher – auch nicht zu Testzwecken.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Bilder herunterladen (Originalgröße), auf ≤ 5 MB JPG/PNG bringen, neutral benennen, Metadaten entfernen.</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Änderungen dokumentieren (CC BY verlangt Hinweis auf Bearbeitung bei Weitergabe).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Je Bild 3 Durchläufe in reason8, jeweils neuer Chat, identische neutrale Instruktion wie im Seminar, gleiches Modell.</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Modell/Version und Datum festhalten; Tool zu t1 und t2 identisch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Rohausgaben unverändert sichern.</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Keine Nachfragen, keine Korrektur.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Kodieren mit vorläufigen Indikatoren: Diagnose-/Ursachenzuschreibung ohne Bildbeleg; Defizit-, Leid- oder Inspirationsvokabular; Hilfsmittel vor Person; Zuschreibung von Alter, Geschlecht, Herkunft, Emotion; Person-first vs. identity-first.</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Bild geeignet, wenn in ≥ 2 von 3 Ausgaben mindestens ein Indikator kodierbar ist (Vorschlag, Schwelle setzen Sie).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Varianz zwischen den 3 Ausgaben notieren.</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Hohe Varianz = Einzelausgaben der Studierenden schwer vergleichbar; im Design berücksichtigen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Ein Bild ohne erwartbare Muster als Kontrast mitlaufen lassen (z. B. Nr. 6).</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Prüft, ob Muster bildgetrieben oder instruktionsgetrieben sind.</t>
         </is>
       </c>
     </row>
@@ -2135,8 +2639,156 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Pilotverfahren</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Schritt</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Inhalt</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Kriterium / Hinweis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Erst nach schriftlicher Rechteklärung (Projekt + HU-DSB) hochladen.</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Kein Upload vorher – auch nicht zu Testzwecken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Bilder herunterladen (Originalgröße), auf ≤ 5 MB JPG/PNG bringen, neutral benennen, Metadaten entfernen.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Änderungen dokumentieren (CC BY verlangt Hinweis auf Bearbeitung bei Weitergabe).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Je Bild 3 Durchläufe in reason8, jeweils neuer Chat, identische neutrale Instruktion wie im Seminar, gleiches Modell.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Modell/Version und Datum festhalten; Tool zu t1 und t2 identisch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Rohausgaben unverändert sichern.</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Keine Nachfragen, keine Korrektur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Kodieren mit vorläufigen Indikatoren: Diagnose-/Ursachenzuschreibung ohne Bildbeleg; Defizit-, Leid- oder Inspirationsvokabular; Hilfsmittel vor Person; Zuschreibung von Alter, Geschlecht, Herkunft, Emotion; Person-first vs. identity-first.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Bild geeignet, wenn in ≥ 2 von 3 Ausgaben mindestens ein Indikator kodierbar ist (Vorschlag, Schwelle setzen Sie).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Varianz zwischen den 3 Ausgaben notieren.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Hohe Varianz = Einzelausgaben der Studierenden schwer vergleichbar; im Design berücksichtigen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Ein Bild ohne erwartbare Muster als Kontrast mitlaufen lassen (z. B. Nr. 6).</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Prüft, ob Muster bildgetrieben oder instruktionsgetrieben sind.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>

</xml_diff>